<commit_message>
update info tab on CSV, added links, added (R) and TM to glossary, amended attenuation grade text throughout project
</commit_message>
<xml_diff>
--- a/assets/program_logic_v6.xlsx
+++ b/assets/program_logic_v6.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7100f48b682a1df6/Work/20251027 IEC TC86 Digital Tool/v3/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7100f48b682a1df6/Work/20251027 IEC TC86 Digital Tool/Digital tool/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="405" documentId="13_ncr:1_{FD3D256E-43A5-4E0A-8438-014B95F3FA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49A7B3DF-464B-4946-8342-81C72661BEA4}"/>
+  <xr:revisionPtr revIDLastSave="438" documentId="13_ncr:1_{FD3D256E-43A5-4E0A-8438-014B95F3FA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{452AD1B3-3213-4E75-A2BF-84455BF5C1ED}"/>
   <bookViews>
-    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="7" xr2:uid="{0D1380F2-B44E-49CB-9379-F623B51E2EAA}"/>
+    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="10" xr2:uid="{0D1380F2-B44E-49CB-9379-F623B51E2EAA}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="8" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="Filter 3" sheetId="16" r:id="rId11"/>
     <sheet name="Filter 4" sheetId="19" r:id="rId12"/>
     <sheet name="Filter 5" sheetId="20" r:id="rId13"/>
+    <sheet name="INFO" sheetId="21" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="182">
   <si>
     <t>Connector type</t>
   </si>
@@ -401,29 +402,282 @@
     <t>IN3</t>
   </si>
   <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Bm</t>
-  </si>
-  <si>
-    <t>Cm</t>
-  </si>
-  <si>
     <t>IN7</t>
   </si>
   <si>
     <t>Mechanical and environmental cable performance</t>
+  </si>
+  <si>
+    <t>Attenuation grade</t>
+  </si>
+  <si>
+    <t>Return loss grade</t>
+  </si>
+  <si>
+    <t>    "IN1": ["LC", "LSH", "MDC", "MPO 1x12", "MPO 1x16", "MPO 2x12", "MPO 2x16", "SAC", "SC", "SEN"],</t>
+  </si>
+  <si>
+    <t>    "IN2": ["Single-mode", "Multimode"],</t>
+  </si>
+  <si>
+    <t>    "IN3": ["Primary coated fibre", "Buffered fibre", "Ribbon fibre", "Reinforced cable"],</t>
+  </si>
+  <si>
+    <t>    "IN4": ["PC", "APC"],</t>
+  </si>
+  <si>
+    <t>    "IN6": ["1 (≥ 60 dB, mated)", "2 (≥ 45 dB, mated)", "3 (≥ 35 dB, mated)", "4 (≥ 26 dB, mated)", "1m (≥ 45 dB, mated)", "2m (≥ 20 dB, mated)"],</t>
+  </si>
+  <si>
+    <t>    "IN7": ["C", "C-HD", "OP", "OP+", "OP+-HD", "OP-HD"]</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Variables in this document must be formatted exactly as follows, as specified in the variable "inputOptions" in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>main.js:</t>
+    </r>
+  </si>
+  <si>
+    <t>    ],</t>
+  </si>
+  <si>
+    <t>    ]</t>
+  </si>
+  <si>
+    <t>"1": [</t>
+  </si>
+  <si>
+    <t>      "Connector type",</t>
+  </si>
+  <si>
+    <t>      "Fibre type",</t>
+  </si>
+  <si>
+    <t>      "PC or APC ferrule end face",</t>
+  </si>
+  <si>
+    <t>      "Attenuation and return loss grades",</t>
+  </si>
+  <si>
+    <t>      "Visual connector end face requirements",</t>
+  </si>
+  <si>
+    <t>      "Connector end face geometric and ferrule parameters",</t>
+  </si>
+  <si>
+    <t>      "Reference connector attenuation requirements",</t>
+  </si>
+  <si>
+    <t>      "Reference connector end face geometric and ferrule parameters"</t>
+  </si>
+  <si>
+    <t>    "2": [</t>
+  </si>
+  <si>
+    <t>      "Mechanical connector interface"</t>
+  </si>
+  <si>
+    <t>    "3": [</t>
+  </si>
+  <si>
+    <t>      "Performance category - operating service environment (temperature range)",</t>
+  </si>
+  <si>
+    <t>      "Mechanical and environmental connector performance (terminated as pigtail or patchcord)"</t>
+  </si>
+  <si>
+    <t>    "4": [</t>
+  </si>
+  <si>
+    <t>      "Cable type",</t>
+  </si>
+  <si>
+    <t>      "Mechanical and environmental cable performance"</t>
+  </si>
+  <si>
+    <t>    "5": [</t>
+  </si>
+  <si>
+    <t>      "Attenuation measurement of randomly mated connectors"</t>
+  </si>
+  <si>
+    <t>    "6": [</t>
+  </si>
+  <si>
+    <t>      "Attenuation and return loss measurement of installed cable plant"</t>
+  </si>
+  <si>
+    <t>    "7": [</t>
+  </si>
+  <si>
+    <t>      "Standard"</t>
+  </si>
+  <si>
+    <t>    "8": [</t>
+  </si>
+  <si>
+    <t>      "Standard",</t>
+  </si>
+  <si>
+    <t>      "Scope"</t>
+  </si>
+  <si>
+    <t>    "Filter 1": [</t>
+  </si>
+  <si>
+    <t>      "IN1",</t>
+  </si>
+  <si>
+    <t>      "IN2",</t>
+  </si>
+  <si>
+    <t>      "IN4"</t>
+  </si>
+  <si>
+    <t>    "Filter 2": [</t>
+  </si>
+  <si>
+    <t>      "IN4",</t>
+  </si>
+  <si>
+    <t>      "IN6"</t>
+  </si>
+  <si>
+    <t>    "Filter 3": [</t>
+  </si>
+  <si>
+    <t>      "IN5",</t>
+  </si>
+  <si>
+    <t>      "IN2"</t>
+  </si>
+  <si>
+    <t>    "Filter 4": [</t>
+  </si>
+  <si>
+    <t>      "IN3",</t>
+  </si>
+  <si>
+    <t>      "IN1"</t>
+  </si>
+  <si>
+    <t>    "Filter 5": [</t>
+  </si>
+  <si>
+    <t>      "IN7"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The headings for each sheet must match exactly those specified in the variable "expectedSheetsAndColumns" in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>main.js:</t>
+    </r>
+  </si>
+  <si>
+    <t>Note 1</t>
+  </si>
+  <si>
+    <t>Note 2</t>
+  </si>
+  <si>
+    <t>Note 3</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">INPUT values are used in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Filter </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">tabs to allow the program to determine which input options are valid in combination with previously selected user inputs. Those are looked up from </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">html </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>id's</t>
+    </r>
+  </si>
+  <si>
+    <t>    "IN5": ["B (mean ≤ 0,12 dB; at least 97 % ≤ 0,25 dB)", "C (mean ≤ 0,25 dB; at least 97 % ≤ 0,5 dB)", "D (mean ≤ 0,5 dB; at least 97 % ≤ 1,0 dB)", "Bm (mean ≤ 0,3 dB; at least 97 % ≤ 0,6 dB)", "Cm (mean ≤ 0,5 dB; at least 97 % ≤ 1,0 dB)"],</t>
+  </si>
+  <si>
+    <t>B (mean ≤ 0,12 dB; at least 97 % ≤ 0,25 dB)</t>
+  </si>
+  <si>
+    <t>C (mean ≤ 0,25 dB; at least 97 % ≤ 0,5 dB)</t>
+  </si>
+  <si>
+    <t>D (mean ≤ 0,5 dB; at least 97 % ≤ 1,0 dB)</t>
+  </si>
+  <si>
+    <t>Bm (mean ≤ 0,3 dB; at least 97 % ≤ 0,6 dB)</t>
+  </si>
+  <si>
+    <t>Cm (mean ≤ 0,5 dB; at least 97 % ≤ 1,0 dB)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -486,8 +740,17 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -524,8 +787,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -533,11 +802,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -611,6 +889,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1837,7 +2118,7 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.42578125" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" style="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="12"/>
@@ -1853,7 +2134,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>117</v>
+        <v>177</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>45</v>
@@ -1861,7 +2142,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>23</v>
+        <v>178</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>45</v>
@@ -1869,7 +2150,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>118</v>
+        <v>179</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>45</v>
@@ -1877,7 +2158,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
-        <v>119</v>
+        <v>180</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>1</v>
@@ -1885,7 +2166,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
-        <v>120</v>
+        <v>181</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>1</v>
@@ -2170,7 +2451,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2205,6 +2486,447 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0B3FE3C-7D18-4B18-A8AC-ABE63533F11D}">
+  <dimension ref="A2:C82"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" style="31"/>
+    <col min="3" max="3" width="68.140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="31"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="B2" s="33" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="31" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="31" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="31" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="31" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="31" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="31" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="32" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="B20" s="33" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="31" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="31" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B25" s="31" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="31" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="31" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="31" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B30" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B31" s="31" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B32" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="31" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="31" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="31" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B37" s="31" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38" s="31" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" s="31" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B41" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B42" s="31" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B43" s="31" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B44" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B45" s="31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B46" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B47" s="31" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B48" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B49" s="31" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" s="31" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B52" s="31" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" s="31" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55" s="31" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" s="31" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" s="31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59" s="31" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60" s="31" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B62" s="31" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B63" s="31" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64" s="31" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65" s="31" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" s="31" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68" s="31" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B69" s="31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B70" s="31" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B71" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B72" s="31" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B73" s="31" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B74" s="31" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B75" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B76" s="31" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B77" s="31" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B78" s="31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B79" s="31" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B80" s="31" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B81" s="31" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B82" s="31" t="s">
+        <v>129</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="271" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2497,7 +3219,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>

</xml_diff>